<commit_message>
chore(data-release): publish site data 2026-09-08 06:07:51 UTC
</commit_message>
<xml_diff>
--- a/diseases/d004/2026-2029.xlsx
+++ b/diseases/d004/2026-2029.xlsx
@@ -29879,13 +29879,13 @@
         </is>
       </c>
       <c r="N177" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="O177" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="R177" t="n">
-        <v>0.05336427512592412</v>
+        <v>0.142304733669131</v>
       </c>
       <c r="S177" t="inlineStr">
         <is>
@@ -30038,10 +30038,10 @@
         </is>
       </c>
       <c r="N178" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="O178" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="U178" t="inlineStr">
         <is>
@@ -30383,7 +30383,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>975486</v>
+        <v>975491</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-09-10 06:22:05 UTC
</commit_message>
<xml_diff>
--- a/diseases/d004/2026-2029.xlsx
+++ b/diseases/d004/2026-2029.xlsx
@@ -27480,13 +27480,13 @@
         </is>
       </c>
       <c r="N161" t="n">
-        <v>9743</v>
+        <v>9744</v>
       </c>
       <c r="O161" t="n">
-        <v>9743</v>
+        <v>9744</v>
       </c>
       <c r="R161" t="n">
-        <v>35.78420555758132</v>
+        <v>35.78787836940084</v>
       </c>
       <c r="S161" t="inlineStr">
         <is>
@@ -30024,13 +30024,13 @@
         </is>
       </c>
       <c r="N178" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="O178" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="R178" t="n">
-        <v>0.2312451922123379</v>
+        <v>0.2668213756296206</v>
       </c>
       <c r="S178" t="inlineStr">
         <is>
@@ -30183,10 +30183,10 @@
         </is>
       </c>
       <c r="N179" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="O179" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="U179" t="inlineStr">
         <is>
@@ -30528,7 +30528,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>980984</v>
+        <v>980987</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-09-12 06:37:19 UTC
</commit_message>
<xml_diff>
--- a/diseases/d004/2026-2029.xlsx
+++ b/diseases/d004/2026-2029.xlsx
@@ -30317,13 +30317,13 @@
         </is>
       </c>
       <c r="N180" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="O180" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="R180" t="n">
-        <v>0.2668213756296206</v>
+        <v>0.3201856507555447</v>
       </c>
       <c r="S180" t="inlineStr">
         <is>
@@ -30476,10 +30476,10 @@
         </is>
       </c>
       <c r="N181" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="O181" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="U181" t="inlineStr">
         <is>
@@ -30821,7 +30821,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1751772</v>
+        <v>1751775</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-09-14 02:13:15 UTC
</commit_message>
<xml_diff>
--- a/diseases/d004/2026-2029.xlsx
+++ b/diseases/d004/2026-2029.xlsx
@@ -27480,13 +27480,13 @@
         </is>
       </c>
       <c r="N161" t="n">
-        <v>9745</v>
+        <v>9749</v>
       </c>
       <c r="O161" t="n">
-        <v>9745</v>
+        <v>9749</v>
       </c>
       <c r="R161" t="n">
-        <v>35.79155118122036</v>
+        <v>35.80624242849844</v>
       </c>
       <c r="S161" t="inlineStr">
         <is>
@@ -30821,7 +30821,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1751775</v>
+        <v>1751779</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-09-16 04:42:23 UTC
</commit_message>
<xml_diff>
--- a/diseases/d004/2026-2029.xlsx
+++ b/diseases/d004/2026-2029.xlsx
@@ -26362,13 +26362,13 @@
         </is>
       </c>
       <c r="N154" t="n">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="O154" t="n">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="R154" t="n">
-        <v>8.870011587752877</v>
+        <v>8.888924192417596</v>
       </c>
       <c r="S154" t="inlineStr">
         <is>
@@ -26521,10 +26521,10 @@
         </is>
       </c>
       <c r="N155" t="n">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="O155" t="n">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="U155" t="inlineStr">
         <is>
@@ -29408,12 +29408,12 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>NZ</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>New Zealand</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -29438,7 +29438,7 @@
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="M174" t="inlineStr">
@@ -29447,56 +29447,70 @@
         </is>
       </c>
       <c r="N174" t="n">
-        <v>6332</v>
+        <v>441</v>
       </c>
       <c r="O174" t="n">
-        <v>6332</v>
+        <v>441</v>
       </c>
       <c r="R174" t="n">
-        <v>5.172030836706432</v>
+        <v>8.340458657140767</v>
       </c>
       <c r="S174" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>SER_NZ_COVID19_MONTHLY</t>
+        </is>
+      </c>
+      <c r="AA174" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO174" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>series_registry</t>
         </is>
       </c>
       <c r="AP174" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR174" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS174" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ174" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS174" t="inlineStr">
+        <is>
+          <t>SER_NZ_COVID19_MONTHLY</t>
+        </is>
+      </c>
       <c r="AT174" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU174" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series.</t>
         </is>
       </c>
       <c r="AV174" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>phf_monthly</t>
         </is>
       </c>
       <c r="AW174" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>New Zealand PHF Science Monthly Notifiable Diseases</t>
         </is>
       </c>
       <c r="AX174" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://www.phfscience.nz/digital-library/</t>
         </is>
       </c>
       <c r="AY174" t="inlineStr">
@@ -29506,17 +29520,17 @@
       </c>
       <c r="AZ174" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>phf_monthly</t>
         </is>
       </c>
       <c r="BA174" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>New Zealand PHF Science Monthly Notifiable Diseases</t>
         </is>
       </c>
       <c r="BB174" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://www.phfscience.nz/digital-library/</t>
         </is>
       </c>
       <c r="BC174" t="inlineStr">
@@ -29548,17 +29562,17 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>NZ</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>New Zealand</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
@@ -29583,7 +29597,7 @@
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="M175" t="inlineStr">
@@ -29592,56 +29606,145 @@
         </is>
       </c>
       <c r="N175" t="n">
-        <v>6578</v>
+        <v>441</v>
       </c>
       <c r="O175" t="n">
-        <v>6578</v>
-      </c>
-      <c r="R175" t="n">
-        <v>5.372965704967611</v>
-      </c>
-      <c r="S175" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
+        <v>441</v>
+      </c>
+      <c r="U175" t="inlineStr">
+        <is>
+          <t>SER_NZ_COVID19_MONTHLY</t>
+        </is>
+      </c>
+      <c r="V175" t="inlineStr">
+        <is>
+          <t>SER_NZ_COVID19_MONTHLY</t>
+        </is>
+      </c>
+      <c r="W175" t="inlineStr">
+        <is>
+          <t>SRC_NZ_PHS</t>
+        </is>
+      </c>
+      <c r="X175" t="inlineStr">
+        <is>
+          <t>COVID-19</t>
+        </is>
+      </c>
+      <c r="Y175" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z175" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA175" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB175" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC175" t="inlineStr">
+        <is>
+          <t>country:NZ:national</t>
+        </is>
+      </c>
+      <c r="AD175" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE175" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF175" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG175" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH175" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI175" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ175" t="inlineStr">
+        <is>
+          <t>NZ_PHS_current</t>
+        </is>
+      </c>
+      <c r="AK175" t="inlineStr">
+        <is>
+          <t>New Zealand PHF Science monthly COVID-19 notifications under the source reporting definition.</t>
+        </is>
+      </c>
+      <c r="AM175" t="inlineStr">
+        <is>
+          <t>provisional; raw</t>
+        </is>
+      </c>
+      <c r="AN175" t="b">
+        <v>1</v>
       </c>
       <c r="AO175" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>series_registry</t>
         </is>
       </c>
       <c r="AP175" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR175" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS175" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ175" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS175" t="inlineStr">
+        <is>
+          <t>SER_NZ_COVID19_MONTHLY</t>
+        </is>
+      </c>
       <c r="AT175" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU175" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series.</t>
         </is>
       </c>
       <c r="AV175" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>phf_monthly</t>
         </is>
       </c>
       <c r="AW175" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>New Zealand PHF Science Monthly Notifiable Diseases</t>
         </is>
       </c>
       <c r="AX175" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://www.phfscience.nz/digital-library/</t>
         </is>
       </c>
       <c r="AY175" t="inlineStr">
@@ -29651,17 +29754,17 @@
       </c>
       <c r="AZ175" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>phf_monthly</t>
         </is>
       </c>
       <c r="BA175" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>New Zealand PHF Science Monthly Notifiable Diseases</t>
         </is>
       </c>
       <c r="BB175" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://www.phfscience.nz/digital-library/</t>
         </is>
       </c>
       <c r="BC175" t="inlineStr">
@@ -29728,7 +29831,7 @@
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="M176" t="inlineStr">
@@ -29737,13 +29840,13 @@
         </is>
       </c>
       <c r="N176" t="n">
-        <v>3896</v>
+        <v>6332</v>
       </c>
       <c r="O176" t="n">
-        <v>3896</v>
+        <v>6332</v>
       </c>
       <c r="R176" t="n">
-        <v>3.182285555876225</v>
+        <v>5.172030836706432</v>
       </c>
       <c r="S176" t="inlineStr">
         <is>
@@ -29873,7 +29976,7 @@
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="M177" t="inlineStr">
@@ -29882,13 +29985,13 @@
         </is>
       </c>
       <c r="N177" t="n">
-        <v>4353</v>
+        <v>6578</v>
       </c>
       <c r="O177" t="n">
-        <v>4353</v>
+        <v>6578</v>
       </c>
       <c r="R177" t="n">
-        <v>3.55556699813378</v>
+        <v>5.372965704967611</v>
       </c>
       <c r="S177" t="inlineStr">
         <is>
@@ -30018,7 +30121,7 @@
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="M178" t="inlineStr">
@@ -30027,13 +30130,13 @@
         </is>
       </c>
       <c r="N178" t="n">
-        <v>5459</v>
+        <v>3896</v>
       </c>
       <c r="O178" t="n">
-        <v>5459</v>
+        <v>3896</v>
       </c>
       <c r="R178" t="n">
-        <v>4.458957096901518</v>
+        <v>3.182285555876225</v>
       </c>
       <c r="S178" t="inlineStr">
         <is>
@@ -30133,12 +30236,12 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
@@ -30163,22 +30266,22 @@
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="N179" t="n">
-        <v>639</v>
+        <v>4353</v>
       </c>
       <c r="O179" t="n">
-        <v>639</v>
+        <v>4353</v>
       </c>
       <c r="R179" t="n">
-        <v>2.346926752673146</v>
+        <v>3.55556699813378</v>
       </c>
       <c r="S179" t="inlineStr">
         <is>
@@ -30211,42 +30314,42 @@
       </c>
       <c r="AV179" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>jp_weekly</t>
         </is>
       </c>
       <c r="AW179" t="inlineStr">
         <is>
-          <t>Australia NINDSS</t>
+          <t>JP NIID Weekly</t>
         </is>
       </c>
       <c r="AX179" t="inlineStr">
         <is>
-          <t>https://www.health.gov.au/topics/national-notifiable-diseases-surveillance-system-nndss</t>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
       <c r="AY179" t="inlineStr">
         <is>
-          <t>microsoft_bi</t>
+          <t>web</t>
         </is>
       </c>
       <c r="AZ179" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>jp_weekly</t>
         </is>
       </c>
       <c r="BA179" t="inlineStr">
         <is>
-          <t>Australia NINDSS</t>
+          <t>JP NIID Weekly</t>
         </is>
       </c>
       <c r="BB179" t="inlineStr">
         <is>
-          <t>https://www.health.gov.au/topics/national-notifiable-diseases-surveillance-system-nndss</t>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
       <c r="BC179" t="inlineStr">
         <is>
-          <t>microsoft_bi</t>
+          <t>web</t>
         </is>
       </c>
     </row>
@@ -30278,12 +30381,12 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
@@ -30308,104 +30411,90 @@
       </c>
       <c r="L180" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="N180" t="n">
-        <v>25</v>
+        <v>5459</v>
       </c>
       <c r="O180" t="n">
-        <v>25</v>
+        <v>5459</v>
       </c>
       <c r="R180" t="n">
-        <v>0.4447022927160344</v>
+        <v>4.458957096901518</v>
       </c>
       <c r="S180" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U180" t="inlineStr">
-        <is>
-          <t>SER_FI_THL_TTR_2801</t>
-        </is>
-      </c>
-      <c r="AA180" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO180" t="inlineStr">
         <is>
-          <t>series_registry</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP180" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ180" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill_blocked_incompatible</t>
-        </is>
-      </c>
-      <c r="AS180" t="inlineStr">
-        <is>
-          <t>SER_FI_THL_TTR_2801</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR180" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS180" t="inlineStr"/>
       <c r="AT180" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU180" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Legacy rows with a different reporting grain or comparison basis were not joined to this curve.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV180" t="inlineStr">
         <is>
-          <t>thl_ttr</t>
+          <t>jp_weekly</t>
         </is>
       </c>
       <c r="AW180" t="inlineStr">
         <is>
-          <t>Finland THL Infectious Diseases Register</t>
+          <t>JP NIID Weekly</t>
         </is>
       </c>
       <c r="AX180" t="inlineStr">
         <is>
-          <t>https://sampo.thl.fi/pivot/prod/en/ttr/cases/fact_ttr_cases</t>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
       <c r="AY180" t="inlineStr">
         <is>
-          <t>cube_csv</t>
+          <t>web</t>
         </is>
       </c>
       <c r="AZ180" t="inlineStr">
         <is>
-          <t>thl_ttr</t>
+          <t>jp_weekly</t>
         </is>
       </c>
       <c r="BA180" t="inlineStr">
         <is>
-          <t>Finland THL Infectious Diseases Register</t>
+          <t>JP NIID Weekly</t>
         </is>
       </c>
       <c r="BB180" t="inlineStr">
         <is>
-          <t>https://sampo.thl.fi/pivot/prod/en/ttr/cases/fact_ttr_cases</t>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
       <c r="BC180" t="inlineStr">
         <is>
-          <t>cube_csv</t>
+          <t>web</t>
         </is>
       </c>
     </row>
@@ -30432,17 +30521,17 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
@@ -30476,170 +30565,81 @@
         </is>
       </c>
       <c r="N181" t="n">
-        <v>25</v>
+        <v>639</v>
       </c>
       <c r="O181" t="n">
-        <v>25</v>
-      </c>
-      <c r="U181" t="inlineStr">
-        <is>
-          <t>SER_FI_THL_TTR_2801</t>
-        </is>
-      </c>
-      <c r="V181" t="inlineStr">
-        <is>
-          <t>SER_FI_THL_TTR_2801</t>
-        </is>
-      </c>
-      <c r="W181" t="inlineStr">
-        <is>
-          <t>SRC_FI_THL_TTR</t>
-        </is>
-      </c>
-      <c r="X181" t="inlineStr">
-        <is>
-          <t>Coronavirus SARS-CoV-2</t>
-        </is>
-      </c>
-      <c r="Y181" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z181" t="inlineStr">
-        <is>
-          <t>national_notifiable_disease_registry</t>
-        </is>
-      </c>
-      <c r="AA181" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="AB181" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC181" t="inlineStr">
-        <is>
-          <t>country:FI:national</t>
-        </is>
-      </c>
-      <c r="AD181" t="inlineStr">
+        <v>639</v>
+      </c>
+      <c r="R181" t="n">
+        <v>2.346926752673146</v>
+      </c>
+      <c r="S181" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO181" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP181" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR181" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS181" t="inlineStr"/>
+      <c r="AT181" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU181" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV181" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="AE181" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF181" t="inlineStr">
-        <is>
-          <t>conditional</t>
-        </is>
-      </c>
-      <c r="AG181" t="inlineStr">
-        <is>
-          <t>non_additive</t>
-        </is>
-      </c>
-      <c r="AH181" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI181" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ181" t="inlineStr">
-        <is>
-          <t>FI_THL_TTR_reporting_group</t>
-        </is>
-      </c>
-      <c r="AK181" t="inlineStr">
-        <is>
-          <t>Finland THL national monthly notification series; THL reporting group code 2801.</t>
-        </is>
-      </c>
-      <c r="AM181" t="inlineStr">
-        <is>
-          <t>provisional; raw</t>
-        </is>
-      </c>
-      <c r="AN181" t="b">
-        <v>1</v>
-      </c>
-      <c r="AO181" t="inlineStr">
-        <is>
-          <t>series_registry</t>
-        </is>
-      </c>
-      <c r="AP181" t="inlineStr">
-        <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ181" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill_blocked_incompatible</t>
-        </is>
-      </c>
-      <c r="AS181" t="inlineStr">
-        <is>
-          <t>SER_FI_THL_TTR_2801</t>
-        </is>
-      </c>
-      <c r="AT181" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU181" t="inlineStr">
-        <is>
-          <t>The public curve is read directly from one registered source series. Legacy rows with a different reporting grain or comparison basis were not joined to this curve.</t>
-        </is>
-      </c>
-      <c r="AV181" t="inlineStr">
-        <is>
-          <t>thl_ttr</t>
-        </is>
-      </c>
       <c r="AW181" t="inlineStr">
         <is>
-          <t>Finland THL Infectious Diseases Register</t>
+          <t>Australia NINDSS</t>
         </is>
       </c>
       <c r="AX181" t="inlineStr">
         <is>
-          <t>https://sampo.thl.fi/pivot/prod/en/ttr/cases/fact_ttr_cases</t>
+          <t>https://www.health.gov.au/topics/national-notifiable-diseases-surveillance-system-nndss</t>
         </is>
       </c>
       <c r="AY181" t="inlineStr">
         <is>
-          <t>cube_csv</t>
+          <t>microsoft_bi</t>
         </is>
       </c>
       <c r="AZ181" t="inlineStr">
         <is>
-          <t>thl_ttr</t>
+          <t>all</t>
         </is>
       </c>
       <c r="BA181" t="inlineStr">
         <is>
-          <t>Finland THL Infectious Diseases Register</t>
+          <t>Australia NINDSS</t>
         </is>
       </c>
       <c r="BB181" t="inlineStr">
         <is>
-          <t>https://sampo.thl.fi/pivot/prod/en/ttr/cases/fact_ttr_cases</t>
+          <t>https://www.health.gov.au/topics/national-notifiable-diseases-surveillance-system-nndss</t>
         </is>
       </c>
       <c r="BC181" t="inlineStr">
         <is>
-          <t>cube_csv</t>
+          <t>microsoft_bi</t>
         </is>
       </c>
     </row>
@@ -30671,118 +30671,511 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
+          <t>FI</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>D004</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>COVID-19</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>新型冠状病毒感染</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N182" t="n">
+        <v>25</v>
+      </c>
+      <c r="O182" t="n">
+        <v>25</v>
+      </c>
+      <c r="R182" t="n">
+        <v>0.4447022927160344</v>
+      </c>
+      <c r="S182" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U182" t="inlineStr">
+        <is>
+          <t>SER_FI_THL_TTR_2801</t>
+        </is>
+      </c>
+      <c r="AA182" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AO182" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP182" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ182" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill_blocked_incompatible</t>
+        </is>
+      </c>
+      <c r="AS182" t="inlineStr">
+        <is>
+          <t>SER_FI_THL_TTR_2801</t>
+        </is>
+      </c>
+      <c r="AT182" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU182" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series. Legacy rows with a different reporting grain or comparison basis were not joined to this curve.</t>
+        </is>
+      </c>
+      <c r="AV182" t="inlineStr">
+        <is>
+          <t>thl_ttr</t>
+        </is>
+      </c>
+      <c r="AW182" t="inlineStr">
+        <is>
+          <t>Finland THL Infectious Diseases Register</t>
+        </is>
+      </c>
+      <c r="AX182" t="inlineStr">
+        <is>
+          <t>https://sampo.thl.fi/pivot/prod/en/ttr/cases/fact_ttr_cases</t>
+        </is>
+      </c>
+      <c r="AY182" t="inlineStr">
+        <is>
+          <t>cube_csv</t>
+        </is>
+      </c>
+      <c r="AZ182" t="inlineStr">
+        <is>
+          <t>thl_ttr</t>
+        </is>
+      </c>
+      <c r="BA182" t="inlineStr">
+        <is>
+          <t>Finland THL Infectious Diseases Register</t>
+        </is>
+      </c>
+      <c r="BB182" t="inlineStr">
+        <is>
+          <t>https://sampo.thl.fi/pivot/prod/en/ttr/cases/fact_ttr_cases</t>
+        </is>
+      </c>
+      <c r="BC182" t="inlineStr">
+        <is>
+          <t>cube_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>disease</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>D004</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>covid-19</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>COVID-19</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>FI</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>D004</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>COVID-19</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>新型冠状病毒感染</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N183" t="n">
+        <v>25</v>
+      </c>
+      <c r="O183" t="n">
+        <v>25</v>
+      </c>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>SER_FI_THL_TTR_2801</t>
+        </is>
+      </c>
+      <c r="V183" t="inlineStr">
+        <is>
+          <t>SER_FI_THL_TTR_2801</t>
+        </is>
+      </c>
+      <c r="W183" t="inlineStr">
+        <is>
+          <t>SRC_FI_THL_TTR</t>
+        </is>
+      </c>
+      <c r="X183" t="inlineStr">
+        <is>
+          <t>Coronavirus SARS-CoV-2</t>
+        </is>
+      </c>
+      <c r="Y183" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z183" t="inlineStr">
+        <is>
+          <t>national_notifiable_disease_registry</t>
+        </is>
+      </c>
+      <c r="AA183" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB183" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC183" t="inlineStr">
+        <is>
+          <t>country:FI:national</t>
+        </is>
+      </c>
+      <c r="AD183" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE183" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF183" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG183" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH183" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI183" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ183" t="inlineStr">
+        <is>
+          <t>FI_THL_TTR_reporting_group</t>
+        </is>
+      </c>
+      <c r="AK183" t="inlineStr">
+        <is>
+          <t>Finland THL national monthly notification series; THL reporting group code 2801.</t>
+        </is>
+      </c>
+      <c r="AM183" t="inlineStr">
+        <is>
+          <t>provisional; raw</t>
+        </is>
+      </c>
+      <c r="AN183" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO183" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP183" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ183" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill_blocked_incompatible</t>
+        </is>
+      </c>
+      <c r="AS183" t="inlineStr">
+        <is>
+          <t>SER_FI_THL_TTR_2801</t>
+        </is>
+      </c>
+      <c r="AT183" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU183" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series. Legacy rows with a different reporting grain or comparison basis were not joined to this curve.</t>
+        </is>
+      </c>
+      <c r="AV183" t="inlineStr">
+        <is>
+          <t>thl_ttr</t>
+        </is>
+      </c>
+      <c r="AW183" t="inlineStr">
+        <is>
+          <t>Finland THL Infectious Diseases Register</t>
+        </is>
+      </c>
+      <c r="AX183" t="inlineStr">
+        <is>
+          <t>https://sampo.thl.fi/pivot/prod/en/ttr/cases/fact_ttr_cases</t>
+        </is>
+      </c>
+      <c r="AY183" t="inlineStr">
+        <is>
+          <t>cube_csv</t>
+        </is>
+      </c>
+      <c r="AZ183" t="inlineStr">
+        <is>
+          <t>thl_ttr</t>
+        </is>
+      </c>
+      <c r="BA183" t="inlineStr">
+        <is>
+          <t>Finland THL Infectious Diseases Register</t>
+        </is>
+      </c>
+      <c r="BB183" t="inlineStr">
+        <is>
+          <t>https://sampo.thl.fi/pivot/prod/en/ttr/cases/fact_ttr_cases</t>
+        </is>
+      </c>
+      <c r="BC183" t="inlineStr">
+        <is>
+          <t>cube_csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>disease</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>D004</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>covid-19</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>COVID-19</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
           <t>JP</t>
         </is>
       </c>
-      <c r="G182" t="inlineStr">
+      <c r="G184" t="inlineStr">
         <is>
           <t>Japan</t>
         </is>
       </c>
-      <c r="H182" t="inlineStr">
-        <is>
-          <t>D004</t>
-        </is>
-      </c>
-      <c r="I182" t="inlineStr">
-        <is>
-          <t>COVID-19</t>
-        </is>
-      </c>
-      <c r="J182" t="inlineStr">
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>D004</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>COVID-19</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
         <is>
           <t>新型冠状病毒感染</t>
         </is>
       </c>
-      <c r="K182" t="inlineStr">
+      <c r="K184" t="inlineStr">
         <is>
           <t>Viral</t>
         </is>
       </c>
-      <c r="L182" t="inlineStr">
+      <c r="L184" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>
       </c>
-      <c r="M182" t="inlineStr">
+      <c r="M184" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="N182" t="n">
+      <c r="N184" t="n">
         <v>7777</v>
       </c>
-      <c r="O182" t="n">
+      <c r="O184" t="n">
         <v>7777</v>
       </c>
-      <c r="R182" t="n">
+      <c r="R184" t="n">
         <v>6.352318985638964</v>
       </c>
-      <c r="S182" t="inlineStr">
+      <c r="S184" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="AO182" t="inlineStr">
+      <c r="AO184" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
         </is>
       </c>
-      <c r="AP182" t="inlineStr">
+      <c r="AP184" t="inlineStr">
         <is>
           <t>legacy_fallback</t>
         </is>
       </c>
-      <c r="AR182" t="inlineStr">
+      <c r="AR184" t="inlineStr">
         <is>
           <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
-      <c r="AS182" t="inlineStr"/>
-      <c r="AT182" t="n">
+      <c r="AS184" t="inlineStr"/>
+      <c r="AT184" t="n">
         <v>0</v>
       </c>
-      <c r="AU182" t="inlineStr">
+      <c r="AU184" t="inlineStr">
         <is>
           <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
-      <c r="AV182" t="inlineStr">
+      <c r="AV184" t="inlineStr">
         <is>
           <t>jp_weekly</t>
         </is>
       </c>
-      <c r="AW182" t="inlineStr">
+      <c r="AW184" t="inlineStr">
         <is>
           <t>JP NIID Weekly</t>
         </is>
       </c>
-      <c r="AX182" t="inlineStr">
+      <c r="AX184" t="inlineStr">
         <is>
           <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
-      <c r="AY182" t="inlineStr">
+      <c r="AY184" t="inlineStr">
         <is>
           <t>web</t>
         </is>
       </c>
-      <c r="AZ182" t="inlineStr">
+      <c r="AZ184" t="inlineStr">
         <is>
           <t>jp_weekly</t>
         </is>
       </c>
-      <c r="BA182" t="inlineStr">
+      <c r="BA184" t="inlineStr">
         <is>
           <t>JP NIID Weekly</t>
         </is>
       </c>
-      <c r="BB182" t="inlineStr">
+      <c r="BB184" t="inlineStr">
         <is>
           <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
-      <c r="BC182" t="inlineStr">
+      <c r="BC184" t="inlineStr">
         <is>
           <t>web</t>
         </is>
@@ -30904,7 +31297,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10">
@@ -30914,7 +31307,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11">
@@ -30934,7 +31327,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13">
@@ -30966,7 +31359,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1759563</v>
+        <v>1760005</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-09-23 04:16:25 UTC
</commit_message>
<xml_diff>
--- a/diseases/d004/2026-2029.xlsx
+++ b/diseases/d004/2026-2029.xlsx
@@ -27480,13 +27480,13 @@
         </is>
       </c>
       <c r="N161" t="n">
-        <v>9749</v>
+        <v>9748</v>
       </c>
       <c r="O161" t="n">
-        <v>9749</v>
+        <v>9748</v>
       </c>
       <c r="R161" t="n">
-        <v>35.80624242849844</v>
+        <v>35.80256961667892</v>
       </c>
       <c r="S161" t="inlineStr">
         <is>
@@ -31359,7 +31359,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1760008</v>
+        <v>1760007</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-10-06 02:14:25 UTC
</commit_message>
<xml_diff>
--- a/diseases/d004/2026-2029.xlsx
+++ b/diseases/d004/2026-2029.xlsx
@@ -41630,13 +41630,13 @@
         </is>
       </c>
       <c r="N238" t="n">
-        <v>7354</v>
+        <v>7379</v>
       </c>
       <c r="O238" t="n">
-        <v>7354</v>
+        <v>7379</v>
       </c>
       <c r="R238" t="n">
-        <v>27.00985812074854</v>
+        <v>27.10167841623653</v>
       </c>
       <c r="S238" t="inlineStr">
         <is>
@@ -43107,7 +43107,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2304477</v>
+        <v>2304502</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-10-06 03:30:29 UTC
</commit_message>
<xml_diff>
--- a/diseases/d004/2026-2029.xlsx
+++ b/diseases/d004/2026-2029.xlsx
@@ -42603,13 +42603,13 @@
         </is>
       </c>
       <c r="N244" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O244" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R244" t="n">
-        <v>0</v>
+        <v>0.1067285502518482</v>
       </c>
       <c r="S244" t="inlineStr">
         <is>
@@ -42762,10 +42762,10 @@
         </is>
       </c>
       <c r="N245" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O245" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U245" t="inlineStr">
         <is>
@@ -43107,7 +43107,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2304502</v>
+        <v>2304508</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-10-13 07:48:52 UTC
</commit_message>
<xml_diff>
--- a/diseases/d004/2026-2029.xlsx
+++ b/diseases/d004/2026-2029.xlsx
@@ -46811,13 +46811,13 @@
         </is>
       </c>
       <c r="N267" t="n">
-        <v>9786</v>
+        <v>9785</v>
       </c>
       <c r="O267" t="n">
-        <v>9786</v>
+        <v>9785</v>
       </c>
       <c r="R267" t="n">
-        <v>35.94213646582067</v>
+        <v>35.93846365400115</v>
       </c>
       <c r="S267" t="inlineStr">
         <is>
@@ -58854,13 +58854,13 @@
         </is>
       </c>
       <c r="N335" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="O335" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="R335" t="n">
-        <v>0.4980665678419585</v>
+        <v>0.6225832098024481</v>
       </c>
       <c r="S335" t="inlineStr">
         <is>
@@ -59013,10 +59013,10 @@
         </is>
       </c>
       <c r="N336" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="O336" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="U336" t="inlineStr">
         <is>
@@ -59358,7 +59358,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2356538</v>
+        <v>2356544</v>
       </c>
     </row>
     <row r="16">

</xml_diff>